<commit_message>
fix: add UTF-8 BOM to CSV files for Excel compatibility
</commit_message>
<xml_diff>
--- a/data/event.xlsx
+++ b/data/event.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10737\Desktop\Planning\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ouyan\课程资料\2026春航天任务分析与设计\航天任务课程实验资料汇总\大作业3\Planning\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0478F1-1876-4A30-A5C2-C67BDCC59FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0603CFEC-8CB8-4930-AB5D-FF7B59D0CE06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>DurationTime(min)</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -52,19 +52,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>备注</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>电能(W）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>约束条件:
-所有编排事件均需避开异常区
-阳光角通过插值计算，满足在约束范围内
-电能约束在某一时刻的上限为1000W
-编排时间窗口为2021-10-02到2021-10-08</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -100,7 +88,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -108,119 +96,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -501,21 +382,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q72"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F72"/>
+  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -526,11 +407,8 @@
       <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="L1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" ht="14" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -549,16 +427,8 @@
       <c r="F2">
         <v>60</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="3"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -577,14 +447,8 @@
       <c r="F3">
         <v>70</v>
       </c>
-      <c r="L3" s="4"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="6"/>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -604,14 +468,8 @@
       <c r="F4">
         <v>20</v>
       </c>
-      <c r="L4" s="4"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="6"/>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>4</v>
       </c>
@@ -630,14 +488,8 @@
       <c r="F5">
         <v>40</v>
       </c>
-      <c r="L5" s="4"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="6"/>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>5</v>
       </c>
@@ -656,14 +508,8 @@
       <c r="F6">
         <v>50</v>
       </c>
-      <c r="L6" s="7"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="9"/>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>6</v>
       </c>
@@ -683,7 +529,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>7</v>
       </c>
@@ -703,7 +549,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>8</v>
       </c>
@@ -723,7 +569,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>9</v>
       </c>
@@ -743,7 +589,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>10</v>
       </c>
@@ -763,7 +609,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>11</v>
       </c>
@@ -783,7 +629,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>12</v>
       </c>
@@ -803,7 +649,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>13</v>
       </c>
@@ -823,7 +669,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>14</v>
       </c>
@@ -843,7 +689,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>15</v>
       </c>
@@ -863,7 +709,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>16</v>
       </c>
@@ -883,7 +729,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>17</v>
       </c>
@@ -903,7 +749,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>18</v>
       </c>
@@ -923,7 +769,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>19</v>
       </c>
@@ -943,7 +789,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>20</v>
       </c>
@@ -963,7 +809,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>21</v>
       </c>
@@ -983,7 +829,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1003,7 +849,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1023,7 +869,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1043,7 +889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1063,7 +909,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1083,7 +929,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1103,7 +949,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1123,7 +969,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1143,7 +989,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1163,7 +1009,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1183,7 +1029,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1203,7 +1049,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1223,7 +1069,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1243,7 +1089,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1263,7 +1109,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1283,7 +1129,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1303,7 +1149,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1323,7 +1169,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1343,7 +1189,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1363,7 +1209,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1383,7 +1229,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1403,7 +1249,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1423,7 +1269,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1443,7 +1289,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1463,7 +1309,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1483,7 +1329,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1503,7 +1349,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1523,7 +1369,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1543,7 +1389,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1563,7 +1409,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1583,7 +1429,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1603,7 +1449,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1623,7 +1469,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1643,7 +1489,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1663,7 +1509,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1683,7 +1529,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1703,7 +1549,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1723,7 +1569,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1743,7 +1589,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1763,7 +1609,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A62">
         <v>61</v>
       </c>
@@ -1783,7 +1629,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A63">
         <v>62</v>
       </c>
@@ -1803,7 +1649,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A64">
         <v>63</v>
       </c>
@@ -1823,7 +1669,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A65">
         <v>64</v>
       </c>
@@ -1843,7 +1689,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A66">
         <v>65</v>
       </c>
@@ -1863,7 +1709,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A67">
         <v>66</v>
       </c>
@@ -1883,7 +1729,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A68">
         <v>67</v>
       </c>
@@ -1903,7 +1749,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A69">
         <v>68</v>
       </c>
@@ -1923,7 +1769,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A70">
         <v>69</v>
       </c>
@@ -1943,7 +1789,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A71">
         <v>70</v>
       </c>
@@ -1963,7 +1809,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A72">
         <v>71</v>
       </c>
@@ -1984,9 +1830,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="L2:Q6"/>
-  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: convert event xlsx to csv and update reader
- Generate event.csv and planningevents.csv from xlsx with corrected
  Chinese headers and resolved formulas
- Replace openpyxl with csv stdlib in main.py
- Update test from workbook mock to csv parse test
</commit_message>
<xml_diff>
--- a/data/event.xlsx
+++ b/data/event.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ouyan\课程资料\2026春航天任务分析与设计\航天任务课程实验资料汇总\大作业3\Planning\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0603CFEC-8CB8-4930-AB5D-FF7B59D0CE06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D869211-AFDF-4DF6-860B-BDF1C4273C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -386,6 +386,10 @@
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">

</xml_diff>